<commit_message>
update .gitignore to exclude .env file
</commit_message>
<xml_diff>
--- a/src/test/resources/datatest/GetProductData.xlsx
+++ b/src/test/resources/datatest/GetProductData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="38">
   <si>
     <t>Product Name</t>
   </si>
@@ -81,6 +81,63 @@
   </si>
   <si>
     <t>25/06/2025 14:40</t>
+  </si>
+  <si>
+    <t>Laptop Asus</t>
+  </si>
+  <si>
+    <t>$3,000.00</t>
+  </si>
+  <si>
+    <t>Aqua, Aquamarine</t>
+  </si>
+  <si>
+    <t>Laptop asus vừa mạnh vừa đẹp</t>
+  </si>
+  <si>
+    <t>https://cms.anhtester.com/public/uploads/all/pM7lRGMTjgwYhP7kB0Zo2FH7ka7OcnpMmjE8DHSk.webp</t>
+  </si>
+  <si>
+    <t>05/07/2025 15:31</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>05/07/2025 16:25</t>
+  </si>
+  <si>
+    <t>05/07/2025 16:36</t>
+  </si>
+  <si>
+    <t>Aqua</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>https://cms.anhtester.com/public/uploads/all/2S6eZZGA1BeFKFx17nPI6L4sxZSdPQG8DMKAm8e1.webp</t>
+  </si>
+  <si>
+    <t>07/07/2025 21:24</t>
+  </si>
+  <si>
+    <t>07/07/2025 21:31</t>
+  </si>
+  <si>
+    <t>07/07/2025 22:00</t>
+  </si>
+  <si>
+    <t>07/07/2025 22:10</t>
+  </si>
+  <si>
+    <t>07/07/2025 22:16</t>
+  </si>
+  <si>
+    <t>07/07/2025 22:22</t>
+  </si>
+  <si>
+    <t>07/07/2025 22:49</t>
   </si>
 </sst>
 </file>
@@ -412,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.296875"/>
@@ -585,6 +642,236 @@
         <v>18</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F16" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Remove .env from Git history
</commit_message>
<xml_diff>
--- a/src/test/resources/datatest/GetProductData.xlsx
+++ b/src/test/resources/datatest/GetProductData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="39">
   <si>
     <t>Product Name</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>07/07/2025 22:49</t>
+  </si>
+  <si>
+    <t>08/07/2025 09:31</t>
   </si>
 </sst>
 </file>
@@ -469,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.296875"/>
@@ -872,6 +875,29 @@
         <v>37</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
remove suite listener file
</commit_message>
<xml_diff>
--- a/src/test/resources/datatest/GetProductData.xlsx
+++ b/src/test/resources/datatest/GetProductData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="40">
   <si>
     <t>Product Name</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>08/07/2025 09:31</t>
+  </si>
+  <si>
+    <t>08/07/2025 09:54</t>
   </si>
 </sst>
 </file>
@@ -472,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.296875"/>
@@ -898,6 +901,29 @@
         <v>38</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update name product search in user add cart test
</commit_message>
<xml_diff>
--- a/src/test/resources/datatest/GetProductData.xlsx
+++ b/src/test/resources/datatest/GetProductData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="43">
   <si>
     <t>Product Name</t>
   </si>
@@ -144,6 +144,15 @@
   </si>
   <si>
     <t>08/07/2025 09:54</t>
+  </si>
+  <si>
+    <t>499</t>
+  </si>
+  <si>
+    <t>10/07/2025 16:01</t>
+  </si>
+  <si>
+    <t>10/07/2025 16:06</t>
   </si>
 </sst>
 </file>
@@ -475,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.296875"/>
@@ -924,6 +933,52 @@
         <v>39</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update 'email from' in EmailUtils
</commit_message>
<xml_diff>
--- a/src/test/resources/datatest/GetProductData.xlsx
+++ b/src/test/resources/datatest/GetProductData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="44">
   <si>
     <t>Product Name</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>10/07/2025 16:06</t>
+  </si>
+  <si>
+    <t>10/07/2025 16:21</t>
   </si>
 </sst>
 </file>
@@ -484,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="14.296875"/>
@@ -979,6 +982,29 @@
         <v>42</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>